<commit_message>
Actualizacion datos REM 2026-09-29 16:13 (orquestador)
</commit_message>
<xml_diff>
--- a/output/reporte_h2_2025.xlsx
+++ b/output/reporte_h2_2025.xlsx
@@ -15,8 +15,8 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Region'!$A$1:$D$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'SS'!$A$1:$E$31</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Comuna'!$A$1:$F$109</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Establecimiento'!$A$1:$G$113</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Comuna'!$A$1:$F$110</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Establecimiento'!$A$1:$G$114</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -494,13 +494,13 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>2275</v>
+        <v>2519</v>
       </c>
       <c r="C2" s="3" t="n">
         <v>4164</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>0.5463496637848223</v>
+        <v>0.6049471661863592</v>
       </c>
     </row>
     <row r="3">
@@ -510,13 +510,13 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>1759</v>
+        <v>1776</v>
       </c>
       <c r="C3" s="3" t="n">
         <v>1886</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>0.9326617179215271</v>
+        <v>0.9416755037115588</v>
       </c>
     </row>
     <row r="4">
@@ -526,13 +526,13 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>1711</v>
+        <v>1743</v>
       </c>
       <c r="C4" s="3" t="n">
         <v>1883</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>0.908656399362719</v>
+        <v>0.9256505576208178</v>
       </c>
     </row>
     <row r="5">
@@ -542,13 +542,13 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>547</v>
+        <v>606</v>
       </c>
       <c r="C5" s="3" t="n">
         <v>700</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>0.7814285714285715</v>
+        <v>0.8657142857142858</v>
       </c>
     </row>
     <row r="6">
@@ -558,13 +558,13 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>6126</v>
+        <v>6231</v>
       </c>
       <c r="C6" s="3" t="n">
         <v>6981</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>0.8775247099269445</v>
+        <v>0.8925655350236356</v>
       </c>
     </row>
     <row r="7">
@@ -574,13 +574,13 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>4463</v>
+        <v>4685</v>
       </c>
       <c r="C7" s="3" t="n">
         <v>5190</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>0.8599229287090558</v>
+        <v>0.9026974951830443</v>
       </c>
     </row>
     <row r="8">
@@ -590,13 +590,13 @@
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>2996</v>
+        <v>3326</v>
       </c>
       <c r="C8" s="3" t="n">
         <v>3873</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>0.7735605473792926</v>
+        <v>0.8587658146139944</v>
       </c>
     </row>
     <row r="9">
@@ -606,13 +606,13 @@
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>3980</v>
+        <v>4162</v>
       </c>
       <c r="C9" s="3" t="n">
         <v>4664</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>0.8533447684391081</v>
+        <v>0.8923670668953688</v>
       </c>
     </row>
     <row r="10">
@@ -622,13 +622,13 @@
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>4548</v>
+        <v>4594</v>
       </c>
       <c r="C10" s="3" t="n">
         <v>4873</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>0.9333059716806895</v>
+        <v>0.9427457418428073</v>
       </c>
     </row>
     <row r="11">
@@ -638,13 +638,13 @@
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>880</v>
+        <v>1041</v>
       </c>
       <c r="C11" s="3" t="n">
         <v>1181</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>0.7451312447078747</v>
+        <v>0.8814563928873835</v>
       </c>
     </row>
     <row r="12">
@@ -654,13 +654,13 @@
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>847</v>
+        <v>856</v>
       </c>
       <c r="C12" s="3" t="n">
         <v>908</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>0.9328193832599119</v>
+        <v>0.9427312775330396</v>
       </c>
     </row>
     <row r="13">
@@ -670,13 +670,13 @@
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>6762</v>
+        <v>6923</v>
       </c>
       <c r="C13" s="3" t="n">
         <v>7572</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>0.893026941362916</v>
+        <v>0.9142894875858426</v>
       </c>
     </row>
     <row r="14">
@@ -686,13 +686,13 @@
         </is>
       </c>
       <c r="B14" s="3" t="n">
-        <v>26062</v>
+        <v>27089</v>
       </c>
       <c r="C14" s="3" t="n">
         <v>29472</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>0.8842969598262758</v>
+        <v>0.9191435939196525</v>
       </c>
     </row>
     <row r="15">
@@ -702,13 +702,13 @@
         </is>
       </c>
       <c r="B15" s="3" t="n">
-        <v>2055</v>
+        <v>2198</v>
       </c>
       <c r="C15" s="3" t="n">
         <v>3213</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>0.6395891690009337</v>
+        <v>0.6840958605664488</v>
       </c>
     </row>
     <row r="16">
@@ -718,13 +718,13 @@
         </is>
       </c>
       <c r="B16" s="3" t="n">
-        <v>3537</v>
+        <v>3636</v>
       </c>
       <c r="C16" s="3" t="n">
         <v>4402</v>
       </c>
       <c r="D16" s="4" t="n">
-        <v>0.803498409813721</v>
+        <v>0.825988187187642</v>
       </c>
     </row>
     <row r="17">
@@ -734,13 +734,13 @@
         </is>
       </c>
       <c r="B17" s="3" t="n">
-        <v>2079</v>
+        <v>2500</v>
       </c>
       <c r="C17" s="3" t="n">
         <v>2487</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>0.8359469240048251</v>
+        <v>1.005227181342984</v>
       </c>
     </row>
   </sheetData>
@@ -804,13 +804,13 @@
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>2275</v>
+        <v>2519</v>
       </c>
       <c r="D2" s="3" t="n">
         <v>4164</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>0.5463496637848223</v>
+        <v>0.6049471661863592</v>
       </c>
     </row>
     <row r="3">
@@ -825,13 +825,13 @@
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>1759</v>
+        <v>1776</v>
       </c>
       <c r="D3" s="3" t="n">
         <v>1886</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>0.9326617179215271</v>
+        <v>0.9416755037115588</v>
       </c>
     </row>
     <row r="4">
@@ -846,13 +846,13 @@
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>1711</v>
+        <v>1743</v>
       </c>
       <c r="D4" s="3" t="n">
         <v>1883</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>0.908656399362719</v>
+        <v>0.9256505576208178</v>
       </c>
     </row>
     <row r="5">
@@ -867,13 +867,13 @@
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>547</v>
+        <v>606</v>
       </c>
       <c r="D5" s="3" t="n">
         <v>700</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>0.7814285714285715</v>
+        <v>0.8657142857142858</v>
       </c>
     </row>
     <row r="6">
@@ -888,13 +888,13 @@
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>712</v>
+        <v>738</v>
       </c>
       <c r="D6" s="3" t="n">
         <v>947</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>0.7518479408658922</v>
+        <v>0.7793030623020063</v>
       </c>
     </row>
     <row r="7">
@@ -909,13 +909,13 @@
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>1938</v>
+        <v>1948</v>
       </c>
       <c r="D7" s="3" t="n">
         <v>2136</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>0.9073033707865169</v>
+        <v>0.9119850187265918</v>
       </c>
     </row>
     <row r="8">
@@ -930,13 +930,13 @@
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>2124</v>
+        <v>2190</v>
       </c>
       <c r="D8" s="3" t="n">
         <v>2453</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>0.8658785161027314</v>
+        <v>0.8927843456991439</v>
       </c>
     </row>
     <row r="9">
@@ -951,13 +951,13 @@
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>1352</v>
+        <v>1355</v>
       </c>
       <c r="D9" s="3" t="n">
         <v>1445</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>0.9356401384083045</v>
+        <v>0.9377162629757786</v>
       </c>
     </row>
     <row r="10">
@@ -972,13 +972,13 @@
         </is>
       </c>
       <c r="C10" s="3" t="n">
-        <v>4463</v>
+        <v>4685</v>
       </c>
       <c r="D10" s="3" t="n">
         <v>5190</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>0.8599229287090558</v>
+        <v>0.9026974951830443</v>
       </c>
     </row>
     <row r="11">
@@ -993,13 +993,13 @@
         </is>
       </c>
       <c r="C11" s="3" t="n">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="D11" s="3" t="n">
         <v>249</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>0.8634538152610441</v>
+        <v>0.8674698795180723</v>
       </c>
     </row>
     <row r="12">
@@ -1014,13 +1014,13 @@
         </is>
       </c>
       <c r="C12" s="3" t="n">
-        <v>2781</v>
+        <v>3110</v>
       </c>
       <c r="D12" s="3" t="n">
         <v>3624</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>0.7673841059602649</v>
+        <v>0.858167770419426</v>
       </c>
     </row>
     <row r="13">
@@ -1035,13 +1035,13 @@
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>3980</v>
+        <v>4162</v>
       </c>
       <c r="D13" s="3" t="n">
         <v>4664</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>0.8533447684391081</v>
+        <v>0.8923670668953688</v>
       </c>
     </row>
     <row r="14">
@@ -1077,13 +1077,13 @@
         </is>
       </c>
       <c r="C15" s="3" t="n">
-        <v>2659</v>
+        <v>2673</v>
       </c>
       <c r="D15" s="3" t="n">
         <v>2749</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>0.9672608221171335</v>
+        <v>0.972353583121135</v>
       </c>
     </row>
     <row r="16">
@@ -1098,13 +1098,13 @@
         </is>
       </c>
       <c r="C16" s="3" t="n">
-        <v>1256</v>
+        <v>1288</v>
       </c>
       <c r="D16" s="3" t="n">
         <v>1445</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>0.8692041522491349</v>
+        <v>0.8913494809688581</v>
       </c>
     </row>
     <row r="17">
@@ -1119,13 +1119,13 @@
         </is>
       </c>
       <c r="C17" s="3" t="n">
-        <v>880</v>
+        <v>1041</v>
       </c>
       <c r="D17" s="3" t="n">
         <v>1181</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>0.7451312447078747</v>
+        <v>0.8814563928873835</v>
       </c>
     </row>
     <row r="18">
@@ -1140,13 +1140,13 @@
         </is>
       </c>
       <c r="C18" s="3" t="n">
-        <v>847</v>
+        <v>856</v>
       </c>
       <c r="D18" s="3" t="n">
         <v>908</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>0.9328193832599119</v>
+        <v>0.9427312775330396</v>
       </c>
     </row>
     <row r="19">
@@ -1161,13 +1161,13 @@
         </is>
       </c>
       <c r="C19" s="3" t="n">
-        <v>6762</v>
+        <v>6923</v>
       </c>
       <c r="D19" s="3" t="n">
         <v>7572</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>0.893026941362916</v>
+        <v>0.9142894875858426</v>
       </c>
     </row>
     <row r="20">
@@ -1203,13 +1203,13 @@
         </is>
       </c>
       <c r="C21" s="3" t="n">
-        <v>3775</v>
+        <v>4151</v>
       </c>
       <c r="D21" s="3" t="n">
         <v>4482</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>0.8422579205711735</v>
+        <v>0.926149040606872</v>
       </c>
     </row>
     <row r="22">
@@ -1224,13 +1224,13 @@
         </is>
       </c>
       <c r="C22" s="3" t="n">
-        <v>6159</v>
+        <v>6637</v>
       </c>
       <c r="D22" s="3" t="n">
         <v>7065</v>
       </c>
       <c r="E22" s="4" t="n">
-        <v>0.8717622080679406</v>
+        <v>0.9394196744515216</v>
       </c>
     </row>
     <row r="23">
@@ -1245,13 +1245,13 @@
         </is>
       </c>
       <c r="C23" s="3" t="n">
-        <v>2559</v>
+        <v>2613</v>
       </c>
       <c r="D23" s="3" t="n">
         <v>2814</v>
       </c>
       <c r="E23" s="4" t="n">
-        <v>0.9093816631130064</v>
+        <v>0.9285714285714286</v>
       </c>
     </row>
     <row r="24">
@@ -1266,13 +1266,13 @@
         </is>
       </c>
       <c r="C24" s="3" t="n">
-        <v>2813</v>
+        <v>2851</v>
       </c>
       <c r="D24" s="3" t="n">
         <v>2938</v>
       </c>
       <c r="E24" s="4" t="n">
-        <v>0.9574540503744043</v>
+        <v>0.9703880190605855</v>
       </c>
     </row>
     <row r="25">
@@ -1287,13 +1287,13 @@
         </is>
       </c>
       <c r="C25" s="3" t="n">
-        <v>5795</v>
+        <v>5876</v>
       </c>
       <c r="D25" s="3" t="n">
         <v>6840</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>0.8472222222222222</v>
+        <v>0.8590643274853801</v>
       </c>
     </row>
     <row r="26">
@@ -1308,13 +1308,13 @@
         </is>
       </c>
       <c r="C26" s="3" t="n">
-        <v>2055</v>
+        <v>2198</v>
       </c>
       <c r="D26" s="3" t="n">
         <v>3213</v>
       </c>
       <c r="E26" s="4" t="n">
-        <v>0.6395891690009337</v>
+        <v>0.6840958605664488</v>
       </c>
     </row>
     <row r="27">
@@ -1329,13 +1329,13 @@
         </is>
       </c>
       <c r="C27" s="3" t="n">
-        <v>1676</v>
+        <v>1747</v>
       </c>
       <c r="D27" s="3" t="n">
         <v>1900</v>
       </c>
       <c r="E27" s="4" t="n">
-        <v>0.8821052631578947</v>
+        <v>0.9194736842105263</v>
       </c>
     </row>
     <row r="28">
@@ -1350,13 +1350,13 @@
         </is>
       </c>
       <c r="C28" s="3" t="n">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="D28" s="3" t="n">
         <v>86</v>
       </c>
       <c r="E28" s="4" t="n">
-        <v>0.8837209302325582</v>
+        <v>0.9418604651162791</v>
       </c>
     </row>
     <row r="29">
@@ -1371,13 +1371,13 @@
         </is>
       </c>
       <c r="C29" s="3" t="n">
-        <v>1784</v>
+        <v>1806</v>
       </c>
       <c r="D29" s="3" t="n">
         <v>2415</v>
       </c>
       <c r="E29" s="4" t="n">
-        <v>0.7387163561076605</v>
+        <v>0.7478260869565218</v>
       </c>
     </row>
     <row r="30">
@@ -1392,13 +1392,13 @@
         </is>
       </c>
       <c r="C30" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D30" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E30" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="31">
@@ -1413,13 +1413,13 @@
         </is>
       </c>
       <c r="C31" s="3" t="n">
-        <v>2079</v>
+        <v>2500</v>
       </c>
       <c r="D31" s="3" t="n">
         <v>2487</v>
       </c>
       <c r="E31" s="4" t="n">
-        <v>0.8359469240048251</v>
+        <v>1.005227181342984</v>
       </c>
     </row>
   </sheetData>
@@ -1434,7 +1434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F109"/>
+  <dimension ref="A1:F110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1494,13 +1494,13 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>1156</v>
+        <v>1176</v>
       </c>
       <c r="E2" s="3" t="n">
         <v>2450</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>0.4718367346938775</v>
+        <v>0.48</v>
       </c>
     </row>
     <row r="3">
@@ -1520,13 +1520,13 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>1073</v>
+        <v>1292</v>
       </c>
       <c r="E3" s="3" t="n">
         <v>1652</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>0.6495157384987893</v>
+        <v>0.7820823244552058</v>
       </c>
     </row>
     <row r="4">
@@ -1546,13 +1546,13 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E4" s="3" t="n">
         <v>11</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>0.09090909090909091</v>
+        <v>0.1818181818181818</v>
       </c>
     </row>
     <row r="5">
@@ -1598,13 +1598,13 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="E6" s="3" t="n">
         <v>10</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>0.9</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="7">
@@ -1650,13 +1650,13 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>1759</v>
+        <v>1776</v>
       </c>
       <c r="E8" s="3" t="n">
         <v>1886</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>0.9326617179215271</v>
+        <v>0.9416755037115588</v>
       </c>
     </row>
     <row r="9">
@@ -1676,13 +1676,13 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E9" s="3" t="n">
         <v>7</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>0.2857142857142857</v>
+        <v>0.5714285714285714</v>
       </c>
     </row>
     <row r="10">
@@ -1702,13 +1702,13 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>1140</v>
+        <v>1170</v>
       </c>
       <c r="E10" s="3" t="n">
         <v>1268</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>0.8990536277602523</v>
+        <v>0.9227129337539433</v>
       </c>
     </row>
     <row r="11">
@@ -1780,13 +1780,13 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E13" s="3" t="n">
         <v>14</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>0.6428571428571429</v>
+        <v>0.7142857142857143</v>
       </c>
     </row>
     <row r="14">
@@ -1832,13 +1832,13 @@
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>538</v>
+        <v>596</v>
       </c>
       <c r="E15" s="3" t="n">
         <v>685</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>0.7854014598540145</v>
+        <v>0.8700729927007299</v>
       </c>
     </row>
     <row r="16">
@@ -1884,13 +1884,13 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>19</v>
+        <v>33</v>
       </c>
       <c r="E17" s="3" t="n">
         <v>28</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>0.6785714285714286</v>
+        <v>1.178571428571429</v>
       </c>
     </row>
     <row r="18">
@@ -1910,13 +1910,13 @@
         </is>
       </c>
       <c r="D18" s="3" t="n">
-        <v>688</v>
+        <v>698</v>
       </c>
       <c r="E18" s="3" t="n">
         <v>909</v>
       </c>
       <c r="F18" s="4" t="n">
-        <v>0.7568756875687569</v>
+        <v>0.7678767876787679</v>
       </c>
     </row>
     <row r="19">
@@ -1936,13 +1936,13 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E19" s="3" t="n">
         <v>9</v>
       </c>
       <c r="F19" s="4" t="n">
-        <v>0.5555555555555556</v>
+        <v>0.7777777777777778</v>
       </c>
     </row>
     <row r="20">
@@ -1962,13 +1962,13 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E20" s="3" t="n">
         <v>6</v>
       </c>
       <c r="F20" s="4" t="n">
-        <v>0.6666666666666666</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21">
@@ -2014,13 +2014,13 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="E22" s="3" t="n">
         <v>10</v>
       </c>
       <c r="F22" s="4" t="n">
-        <v>0.7</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="23">
@@ -2092,13 +2092,13 @@
         </is>
       </c>
       <c r="D25" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E25" s="3" t="n">
         <v>2</v>
       </c>
       <c r="F25" s="4" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26">
@@ -2144,13 +2144,13 @@
         </is>
       </c>
       <c r="D27" s="3" t="n">
-        <v>1640</v>
+        <v>1694</v>
       </c>
       <c r="E27" s="3" t="n">
         <v>1880</v>
       </c>
       <c r="F27" s="4" t="n">
-        <v>0.8723404255319149</v>
+        <v>0.9010638297872341</v>
       </c>
     </row>
     <row r="28">
@@ -2170,13 +2170,13 @@
         </is>
       </c>
       <c r="D28" s="3" t="n">
-        <v>411</v>
+        <v>423</v>
       </c>
       <c r="E28" s="3" t="n">
         <v>495</v>
       </c>
       <c r="F28" s="4" t="n">
-        <v>0.8303030303030303</v>
+        <v>0.8545454545454545</v>
       </c>
     </row>
     <row r="29">
@@ -2274,13 +2274,13 @@
         </is>
       </c>
       <c r="D32" s="3" t="n">
-        <v>1334</v>
+        <v>1336</v>
       </c>
       <c r="E32" s="3" t="n">
         <v>1426</v>
       </c>
       <c r="F32" s="4" t="n">
-        <v>0.9354838709677419</v>
+        <v>0.9368863955119214</v>
       </c>
     </row>
     <row r="33">
@@ -2300,13 +2300,13 @@
         </is>
       </c>
       <c r="D33" s="3" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E33" s="3" t="n">
         <v>15</v>
       </c>
       <c r="F33" s="4" t="n">
-        <v>0.9333333333333333</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34">
@@ -2326,13 +2326,13 @@
         </is>
       </c>
       <c r="D34" s="3" t="n">
-        <v>1545</v>
+        <v>1589</v>
       </c>
       <c r="E34" s="3" t="n">
         <v>1921</v>
       </c>
       <c r="F34" s="4" t="n">
-        <v>0.8042686100989068</v>
+        <v>0.8271733472149921</v>
       </c>
     </row>
     <row r="35">
@@ -2352,13 +2352,13 @@
         </is>
       </c>
       <c r="D35" s="3" t="n">
-        <v>369</v>
+        <v>487</v>
       </c>
       <c r="E35" s="3" t="n">
         <v>429</v>
       </c>
       <c r="F35" s="4" t="n">
-        <v>0.8601398601398601</v>
+        <v>1.135198135198135</v>
       </c>
     </row>
     <row r="36">
@@ -2378,13 +2378,13 @@
         </is>
       </c>
       <c r="D36" s="3" t="n">
-        <v>1389</v>
+        <v>1400</v>
       </c>
       <c r="E36" s="3" t="n">
         <v>1491</v>
       </c>
       <c r="F36" s="4" t="n">
-        <v>0.93158953722334</v>
+        <v>0.9389671361502347</v>
       </c>
     </row>
     <row r="37">
@@ -2430,13 +2430,13 @@
         </is>
       </c>
       <c r="D38" s="3" t="n">
-        <v>1080</v>
+        <v>1122</v>
       </c>
       <c r="E38" s="3" t="n">
         <v>1267</v>
       </c>
       <c r="F38" s="4" t="n">
-        <v>0.8524072612470402</v>
+        <v>0.8855564325177585</v>
       </c>
     </row>
     <row r="39">
@@ -2456,13 +2456,13 @@
         </is>
       </c>
       <c r="D39" s="3" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="E39" s="3" t="n">
         <v>19</v>
       </c>
       <c r="F39" s="4" t="n">
-        <v>1</v>
+        <v>1.315789473684211</v>
       </c>
     </row>
     <row r="40">
@@ -2482,13 +2482,13 @@
         </is>
       </c>
       <c r="D40" s="3" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E40" s="3" t="n">
         <v>18</v>
       </c>
       <c r="F40" s="4" t="n">
-        <v>1</v>
+        <v>1.055555555555556</v>
       </c>
     </row>
     <row r="41">
@@ -2508,13 +2508,13 @@
         </is>
       </c>
       <c r="D41" s="3" t="n">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="E41" s="3" t="n">
         <v>248</v>
       </c>
       <c r="F41" s="4" t="n">
-        <v>0.8669354838709677</v>
+        <v>0.8709677419354839</v>
       </c>
     </row>
     <row r="42">
@@ -2560,13 +2560,13 @@
         </is>
       </c>
       <c r="D43" s="3" t="n">
-        <v>2781</v>
+        <v>3110</v>
       </c>
       <c r="E43" s="3" t="n">
         <v>3624</v>
       </c>
       <c r="F43" s="4" t="n">
-        <v>0.7673841059602649</v>
+        <v>0.858167770419426</v>
       </c>
     </row>
     <row r="44">
@@ -2638,13 +2638,13 @@
         </is>
       </c>
       <c r="D46" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E46" s="3" t="n">
         <v>2</v>
       </c>
       <c r="F46" s="4" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="47">
@@ -2716,13 +2716,13 @@
         </is>
       </c>
       <c r="D49" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E49" s="3" t="n">
         <v>3</v>
       </c>
       <c r="F49" s="4" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.6666666666666666</v>
       </c>
     </row>
     <row r="50">
@@ -2768,13 +2768,13 @@
         </is>
       </c>
       <c r="D51" s="3" t="n">
-        <v>1737</v>
+        <v>1849</v>
       </c>
       <c r="E51" s="3" t="n">
         <v>2125</v>
       </c>
       <c r="F51" s="4" t="n">
-        <v>0.8174117647058824</v>
+        <v>0.8701176470588236</v>
       </c>
     </row>
     <row r="52">
@@ -2794,13 +2794,13 @@
         </is>
       </c>
       <c r="D52" s="3" t="n">
-        <v>792</v>
+        <v>835</v>
       </c>
       <c r="E52" s="3" t="n">
         <v>957</v>
       </c>
       <c r="F52" s="4" t="n">
-        <v>0.8275862068965517</v>
+        <v>0.8725182863113897</v>
       </c>
     </row>
     <row r="53">
@@ -2820,13 +2820,13 @@
         </is>
       </c>
       <c r="D53" s="3" t="n">
-        <v>736</v>
+        <v>743</v>
       </c>
       <c r="E53" s="3" t="n">
         <v>791</v>
       </c>
       <c r="F53" s="4" t="n">
-        <v>0.9304677623261695</v>
+        <v>0.9393173198482933</v>
       </c>
     </row>
     <row r="54">
@@ -2846,13 +2846,13 @@
         </is>
       </c>
       <c r="D54" s="3" t="n">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="E54" s="3" t="n">
         <v>42</v>
       </c>
       <c r="F54" s="4" t="n">
-        <v>0.8809523809523809</v>
+        <v>0.9761904761904762</v>
       </c>
     </row>
     <row r="55">
@@ -2872,13 +2872,13 @@
         </is>
       </c>
       <c r="D55" s="3" t="n">
-        <v>666</v>
+        <v>680</v>
       </c>
       <c r="E55" s="3" t="n">
         <v>725</v>
       </c>
       <c r="F55" s="4" t="n">
-        <v>0.9186206896551724</v>
+        <v>0.9379310344827586</v>
       </c>
     </row>
     <row r="56">
@@ -2924,13 +2924,13 @@
         </is>
       </c>
       <c r="D57" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E57" s="3" t="n">
         <v>6</v>
       </c>
       <c r="F57" s="4" t="n">
-        <v>0.1666666666666667</v>
+        <v>0.3333333333333333</v>
       </c>
     </row>
     <row r="58">
@@ -2998,18 +2998,16 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>Puerto Montt</t>
+          <t>Maullín</t>
         </is>
       </c>
       <c r="D60" s="3" t="n">
-        <v>2654</v>
+        <v>1</v>
       </c>
       <c r="E60" s="3" t="n">
-        <v>2739</v>
-      </c>
-      <c r="F60" s="4" t="n">
-        <v>0.9689667761956918</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F60" s="4" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -3019,22 +3017,22 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>Servicio de Salud Osorno</t>
+          <t>Servicio de Salud Del Reloncaví</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>Osorno</t>
+          <t>Puerto Montt</t>
         </is>
       </c>
       <c r="D61" s="3" t="n">
-        <v>1255</v>
+        <v>2666</v>
       </c>
       <c r="E61" s="3" t="n">
-        <v>1443</v>
+        <v>2739</v>
       </c>
       <c r="F61" s="4" t="n">
-        <v>0.8697158697158697</v>
+        <v>0.9733479372033589</v>
       </c>
     </row>
     <row r="62">
@@ -3050,43 +3048,43 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>Purranque</t>
+          <t>Osorno</t>
         </is>
       </c>
       <c r="D62" s="3" t="n">
-        <v>1</v>
+        <v>1287</v>
       </c>
       <c r="E62" s="3" t="n">
-        <v>2</v>
+        <v>1443</v>
       </c>
       <c r="F62" s="4" t="n">
-        <v>0.5</v>
+        <v>0.8918918918918919</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>Los Ríos</t>
+          <t>Los Lagos</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>Servicio de Salud Los Rios</t>
+          <t>Servicio de Salud Osorno</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>La Unión</t>
+          <t>Purranque</t>
         </is>
       </c>
       <c r="D63" s="3" t="n">
-        <v>64</v>
+        <v>1</v>
       </c>
       <c r="E63" s="3" t="n">
-        <v>70</v>
+        <v>2</v>
       </c>
       <c r="F63" s="4" t="n">
-        <v>0.9142857142857143</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="64">
@@ -3102,17 +3100,17 @@
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>Paillaco</t>
+          <t>La Unión</t>
         </is>
       </c>
       <c r="D64" s="3" t="n">
-        <v>32</v>
+        <v>73</v>
       </c>
       <c r="E64" s="3" t="n">
-        <v>38</v>
+        <v>70</v>
       </c>
       <c r="F64" s="4" t="n">
-        <v>0.8421052631578947</v>
+        <v>1.042857142857143</v>
       </c>
     </row>
     <row r="65">
@@ -3128,17 +3126,17 @@
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>Panguipulli</t>
+          <t>Paillaco</t>
         </is>
       </c>
       <c r="D65" s="3" t="n">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="E65" s="3" t="n">
-        <v>62</v>
+        <v>38</v>
       </c>
       <c r="F65" s="4" t="n">
-        <v>0.7903225806451613</v>
+        <v>1.184210526315789</v>
       </c>
     </row>
     <row r="66">
@@ -3154,17 +3152,17 @@
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>Río Bueno</t>
+          <t>Panguipulli</t>
         </is>
       </c>
       <c r="D66" s="3" t="n">
-        <v>12</v>
+        <v>49</v>
       </c>
       <c r="E66" s="3" t="n">
-        <v>17</v>
+        <v>62</v>
       </c>
       <c r="F66" s="4" t="n">
-        <v>0.7058823529411765</v>
+        <v>0.7903225806451613</v>
       </c>
     </row>
     <row r="67">
@@ -3180,43 +3178,43 @@
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>Valdivia</t>
+          <t>Río Bueno</t>
         </is>
       </c>
       <c r="D67" s="3" t="n">
-        <v>723</v>
+        <v>12</v>
       </c>
       <c r="E67" s="3" t="n">
-        <v>994</v>
+        <v>17</v>
       </c>
       <c r="F67" s="4" t="n">
-        <v>0.727364185110664</v>
+        <v>0.7058823529411765</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>Magallanes y de la Antártica Chilena</t>
+          <t>Los Ríos</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>Servicio de Salud Magallanes</t>
+          <t>Servicio de Salud Los Rios</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>Natales</t>
+          <t>Valdivia</t>
         </is>
       </c>
       <c r="D68" s="3" t="n">
-        <v>161</v>
+        <v>862</v>
       </c>
       <c r="E68" s="3" t="n">
-        <v>174</v>
+        <v>994</v>
       </c>
       <c r="F68" s="4" t="n">
-        <v>0.9252873563218391</v>
+        <v>0.8672032193158954</v>
       </c>
     </row>
     <row r="69">
@@ -3232,17 +3230,17 @@
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>Porvenir</t>
+          <t>Natales</t>
         </is>
       </c>
       <c r="D69" s="3" t="n">
-        <v>1</v>
+        <v>165</v>
       </c>
       <c r="E69" s="3" t="n">
-        <v>2</v>
+        <v>174</v>
       </c>
       <c r="F69" s="4" t="n">
-        <v>0.5</v>
+        <v>0.9482758620689655</v>
       </c>
     </row>
     <row r="70">
@@ -3258,43 +3256,43 @@
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>Punta Arenas</t>
+          <t>Porvenir</t>
         </is>
       </c>
       <c r="D70" s="3" t="n">
-        <v>685</v>
+        <v>2</v>
       </c>
       <c r="E70" s="3" t="n">
-        <v>732</v>
+        <v>2</v>
       </c>
       <c r="F70" s="4" t="n">
-        <v>0.9357923497267759</v>
+        <v>1</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>Maule</t>
+          <t>Magallanes y de la Antártica Chilena</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>Servicio de Salud Del Maule</t>
+          <t>Servicio de Salud Magallanes</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>Cauquenes</t>
+          <t>Punta Arenas</t>
         </is>
       </c>
       <c r="D71" s="3" t="n">
-        <v>160</v>
+        <v>689</v>
       </c>
       <c r="E71" s="3" t="n">
-        <v>188</v>
+        <v>732</v>
       </c>
       <c r="F71" s="4" t="n">
-        <v>0.851063829787234</v>
+        <v>0.9412568306010929</v>
       </c>
     </row>
     <row r="72">
@@ -3310,17 +3308,17 @@
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>Constitución</t>
+          <t>Cauquenes</t>
         </is>
       </c>
       <c r="D72" s="3" t="n">
-        <v>47</v>
+        <v>184</v>
       </c>
       <c r="E72" s="3" t="n">
-        <v>59</v>
+        <v>188</v>
       </c>
       <c r="F72" s="4" t="n">
-        <v>0.7966101694915254</v>
+        <v>0.9787234042553191</v>
       </c>
     </row>
     <row r="73">
@@ -3336,17 +3334,17 @@
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>Curicó</t>
+          <t>Constitución</t>
         </is>
       </c>
       <c r="D73" s="3" t="n">
-        <v>1946</v>
+        <v>71</v>
       </c>
       <c r="E73" s="3" t="n">
-        <v>2062</v>
+        <v>59</v>
       </c>
       <c r="F73" s="4" t="n">
-        <v>0.9437439379243453</v>
+        <v>1.203389830508474</v>
       </c>
     </row>
     <row r="74">
@@ -3362,17 +3360,17 @@
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>Licantén</t>
+          <t>Curicó</t>
         </is>
       </c>
       <c r="D74" s="3" t="n">
-        <v>0</v>
+        <v>1957</v>
       </c>
       <c r="E74" s="3" t="n">
-        <v>3</v>
+        <v>2062</v>
       </c>
       <c r="F74" s="4" t="n">
-        <v>0</v>
+        <v>0.949078564500485</v>
       </c>
     </row>
     <row r="75">
@@ -3388,17 +3386,17 @@
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>Linares</t>
+          <t>Licantén</t>
         </is>
       </c>
       <c r="D75" s="3" t="n">
-        <v>1153</v>
+        <v>1</v>
       </c>
       <c r="E75" s="3" t="n">
-        <v>1437</v>
+        <v>3</v>
       </c>
       <c r="F75" s="4" t="n">
-        <v>0.802366040361865</v>
+        <v>0.3333333333333333</v>
       </c>
     </row>
     <row r="76">
@@ -3414,17 +3412,17 @@
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>Parral</t>
+          <t>Linares</t>
         </is>
       </c>
       <c r="D76" s="3" t="n">
-        <v>71</v>
+        <v>1194</v>
       </c>
       <c r="E76" s="3" t="n">
-        <v>108</v>
+        <v>1437</v>
       </c>
       <c r="F76" s="4" t="n">
-        <v>0.6574074074074074</v>
+        <v>0.8308977035490606</v>
       </c>
     </row>
     <row r="77">
@@ -3440,17 +3438,17 @@
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>San Javier</t>
+          <t>Parral</t>
         </is>
       </c>
       <c r="D77" s="3" t="n">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="E77" s="3" t="n">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="F77" s="4" t="n">
-        <v>0.78</v>
+        <v>0.7592592592592593</v>
       </c>
     </row>
     <row r="78">
@@ -3466,43 +3464,43 @@
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>Talca</t>
+          <t>San Javier</t>
         </is>
       </c>
       <c r="D78" s="3" t="n">
-        <v>3307</v>
+        <v>87</v>
       </c>
       <c r="E78" s="3" t="n">
-        <v>3615</v>
+        <v>100</v>
       </c>
       <c r="F78" s="4" t="n">
-        <v>0.9147994467496542</v>
+        <v>0.87</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>Metropolitana de Santiago</t>
+          <t>Maule</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>Servicio de Salud Metropolitano Central</t>
+          <t>Servicio de Salud Del Maule</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>Maipú</t>
+          <t>Talca</t>
         </is>
       </c>
       <c r="D79" s="3" t="n">
-        <v>2197</v>
+        <v>3347</v>
       </c>
       <c r="E79" s="3" t="n">
-        <v>2305</v>
+        <v>3615</v>
       </c>
       <c r="F79" s="4" t="n">
-        <v>0.9531453362255965</v>
+        <v>0.9258644536652836</v>
       </c>
     </row>
     <row r="80">
@@ -3518,17 +3516,17 @@
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>Santiago</t>
+          <t>Maipú</t>
         </is>
       </c>
       <c r="D80" s="3" t="n">
-        <v>2764</v>
+        <v>2197</v>
       </c>
       <c r="E80" s="3" t="n">
-        <v>3028</v>
+        <v>2305</v>
       </c>
       <c r="F80" s="4" t="n">
-        <v>0.9128137384412153</v>
+        <v>0.9531453362255965</v>
       </c>
     </row>
     <row r="81">
@@ -3539,22 +3537,22 @@
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>Servicio de Salud Metropolitano Norte</t>
+          <t>Servicio de Salud Metropolitano Central</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>Colina</t>
+          <t>Santiago</t>
         </is>
       </c>
       <c r="D81" s="3" t="n">
-        <v>1</v>
+        <v>2764</v>
       </c>
       <c r="E81" s="3" t="n">
-        <v>2</v>
+        <v>3028</v>
       </c>
       <c r="F81" s="4" t="n">
-        <v>0.5</v>
+        <v>0.9128137384412153</v>
       </c>
     </row>
     <row r="82">
@@ -3570,17 +3568,17 @@
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>Independencia</t>
+          <t>Colina</t>
         </is>
       </c>
       <c r="D82" s="3" t="n">
-        <v>3774</v>
+        <v>3</v>
       </c>
       <c r="E82" s="3" t="n">
-        <v>4480</v>
+        <v>2</v>
       </c>
       <c r="F82" s="4" t="n">
-        <v>0.8424107142857142</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="83">
@@ -3591,22 +3589,22 @@
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>Servicio de Salud Metropolitano Occidente</t>
+          <t>Servicio de Salud Metropolitano Norte</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>Cerro Navia</t>
+          <t>Independencia</t>
         </is>
       </c>
       <c r="D83" s="3" t="n">
-        <v>2296</v>
+        <v>4148</v>
       </c>
       <c r="E83" s="3" t="n">
-        <v>2621</v>
+        <v>4480</v>
       </c>
       <c r="F83" s="4" t="n">
-        <v>0.876001526135063</v>
+        <v>0.9258928571428572</v>
       </c>
     </row>
     <row r="84">
@@ -3622,17 +3620,17 @@
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>Curacaví</t>
+          <t>Cerro Navia</t>
         </is>
       </c>
       <c r="D84" s="3" t="n">
-        <v>0</v>
+        <v>2418</v>
       </c>
       <c r="E84" s="3" t="n">
-        <v>1</v>
+        <v>2621</v>
       </c>
       <c r="F84" s="4" t="n">
-        <v>0</v>
+        <v>0.9225486455551316</v>
       </c>
     </row>
     <row r="85">
@@ -3648,17 +3646,17 @@
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>Melipilla</t>
+          <t>Curacaví</t>
         </is>
       </c>
       <c r="D85" s="3" t="n">
-        <v>1281</v>
+        <v>0</v>
       </c>
       <c r="E85" s="3" t="n">
-        <v>1484</v>
+        <v>1</v>
       </c>
       <c r="F85" s="4" t="n">
-        <v>0.8632075471698113</v>
+        <v>0</v>
       </c>
     </row>
     <row r="86">
@@ -3674,17 +3672,17 @@
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>Peñaflor</t>
+          <t>Melipilla</t>
         </is>
       </c>
       <c r="D86" s="3" t="n">
-        <v>52</v>
+        <v>1281</v>
       </c>
       <c r="E86" s="3" t="n">
-        <v>62</v>
+        <v>1484</v>
       </c>
       <c r="F86" s="4" t="n">
-        <v>0.8387096774193549</v>
+        <v>0.8632075471698113</v>
       </c>
     </row>
     <row r="87">
@@ -3700,17 +3698,17 @@
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>Santiago</t>
+          <t>Peñaflor</t>
         </is>
       </c>
       <c r="D87" s="3" t="n">
-        <v>1983</v>
+        <v>52</v>
       </c>
       <c r="E87" s="3" t="n">
-        <v>2072</v>
+        <v>62</v>
       </c>
       <c r="F87" s="4" t="n">
-        <v>0.957046332046332</v>
+        <v>0.8387096774193549</v>
       </c>
     </row>
     <row r="88">
@@ -3726,17 +3724,17 @@
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>Talagante</t>
+          <t>Santiago</t>
         </is>
       </c>
       <c r="D88" s="3" t="n">
-        <v>547</v>
+        <v>2077</v>
       </c>
       <c r="E88" s="3" t="n">
-        <v>825</v>
+        <v>2072</v>
       </c>
       <c r="F88" s="4" t="n">
-        <v>0.6630303030303031</v>
+        <v>1.002413127413127</v>
       </c>
     </row>
     <row r="89">
@@ -3747,22 +3745,22 @@
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>Servicio de Salud Metropolitano Oriente</t>
+          <t>Servicio de Salud Metropolitano Occidente</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>Peñalolén</t>
+          <t>Talagante</t>
         </is>
       </c>
       <c r="D89" s="3" t="n">
-        <v>2559</v>
+        <v>809</v>
       </c>
       <c r="E89" s="3" t="n">
-        <v>2814</v>
+        <v>825</v>
       </c>
       <c r="F89" s="4" t="n">
-        <v>0.9093816631130064</v>
+        <v>0.9806060606060606</v>
       </c>
     </row>
     <row r="90">
@@ -3773,22 +3771,22 @@
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>Servicio de Salud Metropolitano Sur</t>
+          <t>Servicio de Salud Metropolitano Oriente</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>San Bernardo</t>
+          <t>Peñalolén</t>
         </is>
       </c>
       <c r="D90" s="3" t="n">
-        <v>2813</v>
+        <v>2613</v>
       </c>
       <c r="E90" s="3" t="n">
-        <v>2938</v>
+        <v>2814</v>
       </c>
       <c r="F90" s="4" t="n">
-        <v>0.9574540503744043</v>
+        <v>0.9285714285714286</v>
       </c>
     </row>
     <row r="91">
@@ -3799,22 +3797,22 @@
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>Servicio de Salud Metropolitano Sur Oriente</t>
+          <t>Servicio de Salud Metropolitano Sur</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>La Florida</t>
+          <t>San Bernardo</t>
         </is>
       </c>
       <c r="D91" s="3" t="n">
-        <v>1899</v>
+        <v>2851</v>
       </c>
       <c r="E91" s="3" t="n">
-        <v>2045</v>
+        <v>2938</v>
       </c>
       <c r="F91" s="4" t="n">
-        <v>0.9286063569682151</v>
+        <v>0.9703880190605855</v>
       </c>
     </row>
     <row r="92">
@@ -3830,17 +3828,17 @@
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>Puente Alto</t>
+          <t>La Florida</t>
         </is>
       </c>
       <c r="D92" s="3" t="n">
-        <v>2261</v>
+        <v>1908</v>
       </c>
       <c r="E92" s="3" t="n">
-        <v>2941</v>
+        <v>2045</v>
       </c>
       <c r="F92" s="4" t="n">
-        <v>0.7687861271676301</v>
+        <v>0.9330073349633252</v>
       </c>
     </row>
     <row r="93">
@@ -3856,43 +3854,43 @@
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>San Ramón</t>
+          <t>Puente Alto</t>
         </is>
       </c>
       <c r="D93" s="3" t="n">
-        <v>1635</v>
+        <v>2297</v>
       </c>
       <c r="E93" s="3" t="n">
-        <v>1854</v>
+        <v>2941</v>
       </c>
       <c r="F93" s="4" t="n">
-        <v>0.8818770226537217</v>
+        <v>0.7810268616116967</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>Tarapacá</t>
+          <t>Metropolitana de Santiago</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>Servicio de Salud Tarapacá</t>
+          <t>Servicio de Salud Metropolitano Sur Oriente</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>Alto Hospicio</t>
+          <t>San Ramón</t>
         </is>
       </c>
       <c r="D94" s="3" t="n">
-        <v>19</v>
+        <v>1671</v>
       </c>
       <c r="E94" s="3" t="n">
-        <v>21</v>
+        <v>1854</v>
       </c>
       <c r="F94" s="4" t="n">
-        <v>0.9047619047619048</v>
+        <v>0.901294498381877</v>
       </c>
     </row>
     <row r="95">
@@ -3908,43 +3906,43 @@
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>Iquique</t>
+          <t>Alto Hospicio</t>
         </is>
       </c>
       <c r="D95" s="3" t="n">
-        <v>2036</v>
+        <v>23</v>
       </c>
       <c r="E95" s="3" t="n">
-        <v>3192</v>
+        <v>21</v>
       </c>
       <c r="F95" s="4" t="n">
-        <v>0.6378446115288221</v>
+        <v>1.095238095238095</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>Valparaíso</t>
+          <t>Tarapacá</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>Servicio de Salud Aconcagua</t>
+          <t>Servicio de Salud Tarapacá</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>Llaillay</t>
+          <t>Iquique</t>
         </is>
       </c>
       <c r="D96" s="3" t="n">
-        <v>0</v>
+        <v>2175</v>
       </c>
       <c r="E96" s="3" t="n">
-        <v>1</v>
+        <v>3192</v>
       </c>
       <c r="F96" s="4" t="n">
-        <v>0</v>
+        <v>0.681390977443609</v>
       </c>
     </row>
     <row r="97">
@@ -3960,17 +3958,17 @@
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>Los Andes</t>
+          <t>Llaillay</t>
         </is>
       </c>
       <c r="D97" s="3" t="n">
-        <v>627</v>
+        <v>1</v>
       </c>
       <c r="E97" s="3" t="n">
-        <v>637</v>
+        <v>1</v>
       </c>
       <c r="F97" s="4" t="n">
-        <v>0.9843014128728415</v>
+        <v>1</v>
       </c>
     </row>
     <row r="98">
@@ -3986,17 +3984,17 @@
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>San Felipe</t>
+          <t>Los Andes</t>
         </is>
       </c>
       <c r="D98" s="3" t="n">
-        <v>1049</v>
+        <v>630</v>
       </c>
       <c r="E98" s="3" t="n">
-        <v>1262</v>
+        <v>637</v>
       </c>
       <c r="F98" s="4" t="n">
-        <v>0.8312202852614897</v>
+        <v>0.9890109890109891</v>
       </c>
     </row>
     <row r="99">
@@ -4007,22 +4005,22 @@
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>Servicio de Salud Metropolitano Oriente</t>
+          <t>Servicio de Salud Aconcagua</t>
         </is>
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>Isla de Pascua</t>
+          <t>San Felipe</t>
         </is>
       </c>
       <c r="D99" s="3" t="n">
-        <v>76</v>
+        <v>1116</v>
       </c>
       <c r="E99" s="3" t="n">
-        <v>86</v>
+        <v>1262</v>
       </c>
       <c r="F99" s="4" t="n">
-        <v>0.8837209302325582</v>
+        <v>0.884310618066561</v>
       </c>
     </row>
     <row r="100">
@@ -4033,22 +4031,22 @@
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>Servicio de Salud Valparaíso San Antonio</t>
+          <t>Servicio de Salud Metropolitano Oriente</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>San Antonio</t>
+          <t>Isla de Pascua</t>
         </is>
       </c>
       <c r="D100" s="3" t="n">
-        <v>538</v>
+        <v>81</v>
       </c>
       <c r="E100" s="3" t="n">
-        <v>1038</v>
+        <v>86</v>
       </c>
       <c r="F100" s="4" t="n">
-        <v>0.5183044315992292</v>
+        <v>0.9418604651162791</v>
       </c>
     </row>
     <row r="101">
@@ -4064,17 +4062,17 @@
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>Valparaíso</t>
+          <t>San Antonio</t>
         </is>
       </c>
       <c r="D101" s="3" t="n">
-        <v>1246</v>
+        <v>548</v>
       </c>
       <c r="E101" s="3" t="n">
-        <v>1377</v>
+        <v>1038</v>
       </c>
       <c r="F101" s="4" t="n">
-        <v>0.9048656499636892</v>
+        <v>0.5279383429672447</v>
       </c>
     </row>
     <row r="102">
@@ -4085,48 +4083,48 @@
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>Servicio de Salud Viña del Mar Quillota</t>
+          <t>Servicio de Salud Valparaíso San Antonio</t>
         </is>
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>Quintero</t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="D102" s="3" t="n">
-        <v>1</v>
+        <v>1258</v>
       </c>
       <c r="E102" s="3" t="n">
-        <v>1</v>
+        <v>1377</v>
       </c>
       <c r="F102" s="4" t="n">
-        <v>1</v>
+        <v>0.9135802469135802</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>Ñuble</t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>Servicio de Salud Ñuble</t>
+          <t>Servicio de Salud Viña del Mar Quillota</t>
         </is>
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>Bulnes</t>
+          <t>Quintero</t>
         </is>
       </c>
       <c r="D103" s="3" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E103" s="3" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F103" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="104">
@@ -4142,17 +4140,17 @@
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>Chillán</t>
+          <t>Bulnes</t>
         </is>
       </c>
       <c r="D104" s="3" t="n">
-        <v>1544</v>
+        <v>5</v>
       </c>
       <c r="E104" s="3" t="n">
-        <v>1934</v>
+        <v>5</v>
       </c>
       <c r="F104" s="4" t="n">
-        <v>0.7983453981385729</v>
+        <v>1</v>
       </c>
     </row>
     <row r="105">
@@ -4168,17 +4166,17 @@
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>Coelemu</t>
+          <t>Chillán</t>
         </is>
       </c>
       <c r="D105" s="3" t="n">
-        <v>1</v>
+        <v>1748</v>
       </c>
       <c r="E105" s="3" t="n">
-        <v>2</v>
+        <v>1934</v>
       </c>
       <c r="F105" s="4" t="n">
-        <v>0.5</v>
+        <v>0.9038262668045501</v>
       </c>
     </row>
     <row r="106">
@@ -4194,17 +4192,17 @@
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>El Carmen</t>
+          <t>Coelemu</t>
         </is>
       </c>
       <c r="D106" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E106" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F106" s="4" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="107">
@@ -4220,17 +4218,17 @@
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>Quirihue</t>
+          <t>El Carmen</t>
         </is>
       </c>
       <c r="D107" s="3" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E107" s="3" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F107" s="4" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="108">
@@ -4246,17 +4244,17 @@
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>San Carlos</t>
+          <t>Quirihue</t>
         </is>
       </c>
       <c r="D108" s="3" t="n">
-        <v>526</v>
+        <v>3</v>
       </c>
       <c r="E108" s="3" t="n">
-        <v>538</v>
+        <v>6</v>
       </c>
       <c r="F108" s="4" t="n">
-        <v>0.9776951672862454</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="109">
@@ -4272,21 +4270,47 @@
       </c>
       <c r="C109" s="2" t="inlineStr">
         <is>
+          <t>San Carlos</t>
+        </is>
+      </c>
+      <c r="D109" s="3" t="n">
+        <v>742</v>
+      </c>
+      <c r="E109" s="3" t="n">
+        <v>538</v>
+      </c>
+      <c r="F109" s="4" t="n">
+        <v>1.379182156133829</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>Ñuble</t>
+        </is>
+      </c>
+      <c r="B110" s="2" t="inlineStr">
+        <is>
+          <t>Servicio de Salud Ñuble</t>
+        </is>
+      </c>
+      <c r="C110" s="2" t="inlineStr">
+        <is>
           <t>Yungay</t>
         </is>
       </c>
-      <c r="D109" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E109" s="3" t="n">
+      <c r="D110" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="F109" s="4" t="n">
-        <v>0</v>
+      <c r="E110" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F110" s="4" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F109"/>
+  <autoFilter ref="A1:F110"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4297,7 +4321,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G113"/>
+  <dimension ref="A1:G114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -4368,13 +4392,13 @@
         </is>
       </c>
       <c r="E2" s="3" t="n">
-        <v>1156</v>
+        <v>1176</v>
       </c>
       <c r="F2" s="3" t="n">
         <v>2450</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>0.4718367346938775</v>
+        <v>0.48</v>
       </c>
     </row>
     <row r="3">
@@ -4399,13 +4423,13 @@
         </is>
       </c>
       <c r="E3" s="3" t="n">
-        <v>1073</v>
+        <v>1292</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>1652</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>0.6495157384987893</v>
+        <v>0.7820823244552058</v>
       </c>
     </row>
     <row r="4">
@@ -4430,13 +4454,13 @@
         </is>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F4" s="3" t="n">
         <v>11</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>0.09090909090909091</v>
+        <v>0.1818181818181818</v>
       </c>
     </row>
     <row r="5">
@@ -4492,13 +4516,13 @@
         </is>
       </c>
       <c r="E6" s="3" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="F6" s="3" t="n">
         <v>10</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>0.9</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="7">
@@ -4554,13 +4578,13 @@
         </is>
       </c>
       <c r="E8" s="3" t="n">
-        <v>1759</v>
+        <v>1776</v>
       </c>
       <c r="F8" s="3" t="n">
         <v>1886</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>0.9326617179215271</v>
+        <v>0.9416755037115588</v>
       </c>
     </row>
     <row r="9">
@@ -4585,13 +4609,13 @@
         </is>
       </c>
       <c r="E9" s="3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F9" s="3" t="n">
         <v>7</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>0.2857142857142857</v>
+        <v>0.5714285714285714</v>
       </c>
     </row>
     <row r="10">
@@ -4616,13 +4640,13 @@
         </is>
       </c>
       <c r="E10" s="3" t="n">
-        <v>1140</v>
+        <v>1170</v>
       </c>
       <c r="F10" s="3" t="n">
         <v>1268</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>0.8990536277602523</v>
+        <v>0.9227129337539433</v>
       </c>
     </row>
     <row r="11">
@@ -4709,13 +4733,13 @@
         </is>
       </c>
       <c r="E13" s="3" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F13" s="3" t="n">
         <v>14</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>0.6428571428571429</v>
+        <v>0.7142857142857143</v>
       </c>
     </row>
     <row r="14">
@@ -4771,13 +4795,13 @@
         </is>
       </c>
       <c r="E15" s="3" t="n">
-        <v>538</v>
+        <v>596</v>
       </c>
       <c r="F15" s="3" t="n">
         <v>685</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>0.7854014598540145</v>
+        <v>0.8700729927007299</v>
       </c>
     </row>
     <row r="16">
@@ -4833,13 +4857,13 @@
         </is>
       </c>
       <c r="E17" s="3" t="n">
-        <v>19</v>
+        <v>33</v>
       </c>
       <c r="F17" s="3" t="n">
         <v>28</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>0.6785714285714286</v>
+        <v>1.178571428571429</v>
       </c>
     </row>
     <row r="18">
@@ -4864,13 +4888,13 @@
         </is>
       </c>
       <c r="E18" s="3" t="n">
-        <v>688</v>
+        <v>698</v>
       </c>
       <c r="F18" s="3" t="n">
         <v>909</v>
       </c>
       <c r="G18" s="4" t="n">
-        <v>0.7568756875687569</v>
+        <v>0.7678767876787679</v>
       </c>
     </row>
     <row r="19">
@@ -4895,13 +4919,13 @@
         </is>
       </c>
       <c r="E19" s="3" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F19" s="3" t="n">
         <v>9</v>
       </c>
       <c r="G19" s="4" t="n">
-        <v>0.5555555555555556</v>
+        <v>0.7777777777777778</v>
       </c>
     </row>
     <row r="20">
@@ -4926,13 +4950,13 @@
         </is>
       </c>
       <c r="E20" s="3" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F20" s="3" t="n">
         <v>6</v>
       </c>
       <c r="G20" s="4" t="n">
-        <v>0.6666666666666666</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21">
@@ -4988,13 +5012,13 @@
         </is>
       </c>
       <c r="E22" s="3" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="F22" s="3" t="n">
         <v>10</v>
       </c>
       <c r="G22" s="4" t="n">
-        <v>0.7</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="23">
@@ -5081,13 +5105,13 @@
         </is>
       </c>
       <c r="E25" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F25" s="3" t="n">
         <v>2</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26">
@@ -5143,13 +5167,13 @@
         </is>
       </c>
       <c r="E27" s="3" t="n">
-        <v>1640</v>
+        <v>1694</v>
       </c>
       <c r="F27" s="3" t="n">
         <v>1880</v>
       </c>
       <c r="G27" s="4" t="n">
-        <v>0.8723404255319149</v>
+        <v>0.9010638297872341</v>
       </c>
     </row>
     <row r="28">
@@ -5174,13 +5198,13 @@
         </is>
       </c>
       <c r="E28" s="3" t="n">
-        <v>411</v>
+        <v>423</v>
       </c>
       <c r="F28" s="3" t="n">
         <v>495</v>
       </c>
       <c r="G28" s="4" t="n">
-        <v>0.8303030303030303</v>
+        <v>0.8545454545454545</v>
       </c>
     </row>
     <row r="29">
@@ -5298,13 +5322,13 @@
         </is>
       </c>
       <c r="E32" s="3" t="n">
-        <v>1334</v>
+        <v>1336</v>
       </c>
       <c r="F32" s="3" t="n">
         <v>1426</v>
       </c>
       <c r="G32" s="4" t="n">
-        <v>0.9354838709677419</v>
+        <v>0.9368863955119214</v>
       </c>
     </row>
     <row r="33">
@@ -5329,13 +5353,13 @@
         </is>
       </c>
       <c r="E33" s="3" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F33" s="3" t="n">
         <v>15</v>
       </c>
       <c r="G33" s="4" t="n">
-        <v>0.9333333333333333</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34">
@@ -5360,13 +5384,13 @@
         </is>
       </c>
       <c r="E34" s="3" t="n">
-        <v>1545</v>
+        <v>1589</v>
       </c>
       <c r="F34" s="3" t="n">
         <v>1921</v>
       </c>
       <c r="G34" s="4" t="n">
-        <v>0.8042686100989068</v>
+        <v>0.8271733472149921</v>
       </c>
     </row>
     <row r="35">
@@ -5391,13 +5415,13 @@
         </is>
       </c>
       <c r="E35" s="3" t="n">
-        <v>369</v>
+        <v>487</v>
       </c>
       <c r="F35" s="3" t="n">
         <v>429</v>
       </c>
       <c r="G35" s="4" t="n">
-        <v>0.8601398601398601</v>
+        <v>1.135198135198135</v>
       </c>
     </row>
     <row r="36">
@@ -5422,13 +5446,13 @@
         </is>
       </c>
       <c r="E36" s="3" t="n">
-        <v>1389</v>
+        <v>1400</v>
       </c>
       <c r="F36" s="3" t="n">
         <v>1491</v>
       </c>
       <c r="G36" s="4" t="n">
-        <v>0.93158953722334</v>
+        <v>0.9389671361502347</v>
       </c>
     </row>
     <row r="37">
@@ -5484,13 +5508,13 @@
         </is>
       </c>
       <c r="E38" s="3" t="n">
-        <v>1080</v>
+        <v>1122</v>
       </c>
       <c r="F38" s="3" t="n">
         <v>1267</v>
       </c>
       <c r="G38" s="4" t="n">
-        <v>0.8524072612470402</v>
+        <v>0.8855564325177585</v>
       </c>
     </row>
     <row r="39">
@@ -5515,13 +5539,13 @@
         </is>
       </c>
       <c r="E39" s="3" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="F39" s="3" t="n">
         <v>19</v>
       </c>
       <c r="G39" s="4" t="n">
-        <v>1</v>
+        <v>1.315789473684211</v>
       </c>
     </row>
     <row r="40">
@@ -5546,13 +5570,13 @@
         </is>
       </c>
       <c r="E40" s="3" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F40" s="3" t="n">
         <v>18</v>
       </c>
       <c r="G40" s="4" t="n">
-        <v>1</v>
+        <v>1.055555555555556</v>
       </c>
     </row>
     <row r="41">
@@ -5577,13 +5601,13 @@
         </is>
       </c>
       <c r="E41" s="3" t="n">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="F41" s="3" t="n">
         <v>248</v>
       </c>
       <c r="G41" s="4" t="n">
-        <v>0.8669354838709677</v>
+        <v>0.8709677419354839</v>
       </c>
     </row>
     <row r="42">
@@ -5639,13 +5663,13 @@
         </is>
       </c>
       <c r="E43" s="3" t="n">
-        <v>2781</v>
+        <v>3110</v>
       </c>
       <c r="F43" s="3" t="n">
         <v>3624</v>
       </c>
       <c r="G43" s="4" t="n">
-        <v>0.7673841059602649</v>
+        <v>0.858167770419426</v>
       </c>
     </row>
     <row r="44">
@@ -5732,13 +5756,13 @@
         </is>
       </c>
       <c r="E46" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F46" s="3" t="n">
         <v>2</v>
       </c>
       <c r="G46" s="4" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="47">
@@ -5825,13 +5849,13 @@
         </is>
       </c>
       <c r="E49" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F49" s="3" t="n">
         <v>3</v>
       </c>
       <c r="G49" s="4" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.6666666666666666</v>
       </c>
     </row>
     <row r="50">
@@ -5887,13 +5911,13 @@
         </is>
       </c>
       <c r="E51" s="3" t="n">
-        <v>1737</v>
+        <v>1849</v>
       </c>
       <c r="F51" s="3" t="n">
         <v>2125</v>
       </c>
       <c r="G51" s="4" t="n">
-        <v>0.8174117647058824</v>
+        <v>0.8701176470588236</v>
       </c>
     </row>
     <row r="52">
@@ -5918,13 +5942,13 @@
         </is>
       </c>
       <c r="E52" s="3" t="n">
-        <v>792</v>
+        <v>835</v>
       </c>
       <c r="F52" s="3" t="n">
         <v>957</v>
       </c>
       <c r="G52" s="4" t="n">
-        <v>0.8275862068965517</v>
+        <v>0.8725182863113897</v>
       </c>
     </row>
     <row r="53">
@@ -5980,13 +6004,13 @@
         </is>
       </c>
       <c r="E54" s="3" t="n">
-        <v>735</v>
+        <v>742</v>
       </c>
       <c r="F54" s="3" t="n">
         <v>790</v>
       </c>
       <c r="G54" s="4" t="n">
-        <v>0.930379746835443</v>
+        <v>0.9392405063291139</v>
       </c>
     </row>
     <row r="55">
@@ -6011,13 +6035,13 @@
         </is>
       </c>
       <c r="E55" s="3" t="n">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="F55" s="3" t="n">
         <v>42</v>
       </c>
       <c r="G55" s="4" t="n">
-        <v>0.8809523809523809</v>
+        <v>0.9761904761904762</v>
       </c>
     </row>
     <row r="56">
@@ -6042,13 +6066,13 @@
         </is>
       </c>
       <c r="E56" s="3" t="n">
-        <v>666</v>
+        <v>680</v>
       </c>
       <c r="F56" s="3" t="n">
         <v>725</v>
       </c>
       <c r="G56" s="4" t="n">
-        <v>0.9186206896551724</v>
+        <v>0.9379310344827586</v>
       </c>
     </row>
     <row r="57">
@@ -6104,13 +6128,13 @@
         </is>
       </c>
       <c r="E58" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F58" s="3" t="n">
         <v>6</v>
       </c>
       <c r="G58" s="4" t="n">
-        <v>0.1666666666666667</v>
+        <v>0.3333333333333333</v>
       </c>
     </row>
     <row r="59">
@@ -6188,23 +6212,21 @@
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>Puerto Montt</t>
+          <t>Maullín</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>Hospital de Puerto Montt</t>
+          <t>Hospital de Maullín</t>
         </is>
       </c>
       <c r="E61" s="3" t="n">
-        <v>2654</v>
+        <v>1</v>
       </c>
       <c r="F61" s="3" t="n">
-        <v>2739</v>
-      </c>
-      <c r="G61" s="4" t="n">
-        <v>0.9689667761956918</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G61" s="4" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -6214,27 +6236,27 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Servicio de Salud Osorno</t>
+          <t>Servicio de Salud Del Reloncaví</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>Osorno</t>
+          <t>Puerto Montt</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Hospital Base San José de Osorno</t>
+          <t>Hospital de Puerto Montt</t>
         </is>
       </c>
       <c r="E62" s="3" t="n">
-        <v>1255</v>
+        <v>2666</v>
       </c>
       <c r="F62" s="3" t="n">
-        <v>1443</v>
+        <v>2739</v>
       </c>
       <c r="G62" s="4" t="n">
-        <v>0.8697158697158697</v>
+        <v>0.9733479372033589</v>
       </c>
     </row>
     <row r="63">
@@ -6250,53 +6272,53 @@
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>Purranque</t>
+          <t>Osorno</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>Hospital de Purranque Dr. Juan Hepp Dubiau</t>
+          <t>Hospital Base San José de Osorno</t>
         </is>
       </c>
       <c r="E63" s="3" t="n">
-        <v>1</v>
+        <v>1287</v>
       </c>
       <c r="F63" s="3" t="n">
-        <v>2</v>
+        <v>1443</v>
       </c>
       <c r="G63" s="4" t="n">
-        <v>0.5</v>
+        <v>0.8918918918918919</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>Los Ríos</t>
+          <t>Los Lagos</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Servicio de Salud Los Rios</t>
+          <t>Servicio de Salud Osorno</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>La Unión</t>
+          <t>Purranque</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Hospital Juan Morey (La Unión)</t>
+          <t>Hospital de Purranque Dr. Juan Hepp Dubiau</t>
         </is>
       </c>
       <c r="E64" s="3" t="n">
-        <v>64</v>
+        <v>1</v>
       </c>
       <c r="F64" s="3" t="n">
-        <v>70</v>
+        <v>2</v>
       </c>
       <c r="G64" s="4" t="n">
-        <v>0.9142857142857143</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="65">
@@ -6312,22 +6334,22 @@
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>Paillaco</t>
+          <t>La Unión</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>Hospital de Paillaco</t>
+          <t>Hospital Juan Morey (La Unión)</t>
         </is>
       </c>
       <c r="E65" s="3" t="n">
-        <v>32</v>
+        <v>73</v>
       </c>
       <c r="F65" s="3" t="n">
-        <v>38</v>
+        <v>70</v>
       </c>
       <c r="G65" s="4" t="n">
-        <v>0.8421052631578947</v>
+        <v>1.042857142857143</v>
       </c>
     </row>
     <row r="66">
@@ -6343,22 +6365,22 @@
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>Panguipulli</t>
+          <t>Paillaco</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>Hospital de Panguipulli</t>
+          <t>Hospital de Paillaco</t>
         </is>
       </c>
       <c r="E66" s="3" t="n">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="F66" s="3" t="n">
-        <v>62</v>
+        <v>38</v>
       </c>
       <c r="G66" s="4" t="n">
-        <v>0.7903225806451613</v>
+        <v>1.184210526315789</v>
       </c>
     </row>
     <row r="67">
@@ -6374,22 +6396,22 @@
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>Río Bueno</t>
+          <t>Panguipulli</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>Hospital de Río Bueno</t>
+          <t>Hospital de Panguipulli</t>
         </is>
       </c>
       <c r="E67" s="3" t="n">
-        <v>12</v>
+        <v>49</v>
       </c>
       <c r="F67" s="3" t="n">
-        <v>17</v>
+        <v>62</v>
       </c>
       <c r="G67" s="4" t="n">
-        <v>0.7058823529411765</v>
+        <v>0.7903225806451613</v>
       </c>
     </row>
     <row r="68">
@@ -6405,53 +6427,53 @@
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>Valdivia</t>
+          <t>Río Bueno</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>Hospital Base Valdivia</t>
+          <t>Hospital de Río Bueno</t>
         </is>
       </c>
       <c r="E68" s="3" t="n">
-        <v>723</v>
+        <v>12</v>
       </c>
       <c r="F68" s="3" t="n">
-        <v>994</v>
+        <v>17</v>
       </c>
       <c r="G68" s="4" t="n">
-        <v>0.727364185110664</v>
+        <v>0.7058823529411765</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>Magallanes y de la Antártica Chilena</t>
+          <t>Los Ríos</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>Servicio de Salud Magallanes</t>
+          <t>Servicio de Salud Los Rios</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>Natales</t>
+          <t>Valdivia</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>Hospital Dr. Augusto Essmann Burgos ( Natales)</t>
+          <t>Hospital Base Valdivia</t>
         </is>
       </c>
       <c r="E69" s="3" t="n">
-        <v>161</v>
+        <v>862</v>
       </c>
       <c r="F69" s="3" t="n">
-        <v>174</v>
+        <v>994</v>
       </c>
       <c r="G69" s="4" t="n">
-        <v>0.9252873563218391</v>
+        <v>0.8672032193158954</v>
       </c>
     </row>
     <row r="70">
@@ -6467,22 +6489,22 @@
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>Porvenir</t>
+          <t>Natales</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>Hospital Dr. Marco Antonio Chamorro ( Porvenir)</t>
+          <t>Hospital Dr. Augusto Essmann Burgos ( Natales)</t>
         </is>
       </c>
       <c r="E70" s="3" t="n">
-        <v>1</v>
+        <v>165</v>
       </c>
       <c r="F70" s="3" t="n">
-        <v>2</v>
+        <v>174</v>
       </c>
       <c r="G70" s="4" t="n">
-        <v>0.5</v>
+        <v>0.9482758620689655</v>
       </c>
     </row>
     <row r="71">
@@ -6498,53 +6520,53 @@
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>Punta Arenas</t>
+          <t>Porvenir</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>Hospital Clínico de Magallanes Dr. Lautaro Navarro Avaria</t>
+          <t>Hospital Dr. Marco Antonio Chamorro ( Porvenir)</t>
         </is>
       </c>
       <c r="E71" s="3" t="n">
-        <v>685</v>
+        <v>2</v>
       </c>
       <c r="F71" s="3" t="n">
-        <v>732</v>
+        <v>2</v>
       </c>
       <c r="G71" s="4" t="n">
-        <v>0.9357923497267759</v>
+        <v>1</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>Maule</t>
+          <t>Magallanes y de la Antártica Chilena</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>Servicio de Salud Del Maule</t>
+          <t>Servicio de Salud Magallanes</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>Cauquenes</t>
+          <t>Punta Arenas</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>Hospital San Juan de Dios (Cauquenes)</t>
+          <t>Hospital Clínico de Magallanes Dr. Lautaro Navarro Avaria</t>
         </is>
       </c>
       <c r="E72" s="3" t="n">
-        <v>160</v>
+        <v>689</v>
       </c>
       <c r="F72" s="3" t="n">
-        <v>188</v>
+        <v>732</v>
       </c>
       <c r="G72" s="4" t="n">
-        <v>0.851063829787234</v>
+        <v>0.9412568306010929</v>
       </c>
     </row>
     <row r="73">
@@ -6560,22 +6582,22 @@
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>Constitución</t>
+          <t>Cauquenes</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>Hospital de Constitución</t>
+          <t>Hospital San Juan de Dios (Cauquenes)</t>
         </is>
       </c>
       <c r="E73" s="3" t="n">
-        <v>47</v>
+        <v>184</v>
       </c>
       <c r="F73" s="3" t="n">
-        <v>59</v>
+        <v>188</v>
       </c>
       <c r="G73" s="4" t="n">
-        <v>0.7966101694915254</v>
+        <v>0.9787234042553191</v>
       </c>
     </row>
     <row r="74">
@@ -6591,22 +6613,22 @@
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>Curicó</t>
+          <t>Constitución</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>Hospital San Juan de Dios (Curicó)</t>
+          <t>Hospital de Constitución</t>
         </is>
       </c>
       <c r="E74" s="3" t="n">
-        <v>1946</v>
+        <v>71</v>
       </c>
       <c r="F74" s="3" t="n">
-        <v>2062</v>
+        <v>59</v>
       </c>
       <c r="G74" s="4" t="n">
-        <v>0.9437439379243453</v>
+        <v>1.203389830508474</v>
       </c>
     </row>
     <row r="75">
@@ -6622,22 +6644,22 @@
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>Licantén</t>
+          <t>Curicó</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>Hospital de Licantén</t>
+          <t>Hospital San Juan de Dios (Curicó)</t>
         </is>
       </c>
       <c r="E75" s="3" t="n">
-        <v>0</v>
+        <v>1957</v>
       </c>
       <c r="F75" s="3" t="n">
-        <v>3</v>
+        <v>2062</v>
       </c>
       <c r="G75" s="4" t="n">
-        <v>0</v>
+        <v>0.949078564500485</v>
       </c>
     </row>
     <row r="76">
@@ -6653,22 +6675,22 @@
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>Linares</t>
+          <t>Licantén</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>Hospital Presidente Carlos Ibáñez del Campo (Linares)</t>
+          <t>Hospital de Licantén</t>
         </is>
       </c>
       <c r="E76" s="3" t="n">
-        <v>1153</v>
+        <v>1</v>
       </c>
       <c r="F76" s="3" t="n">
-        <v>1437</v>
+        <v>3</v>
       </c>
       <c r="G76" s="4" t="n">
-        <v>0.802366040361865</v>
+        <v>0.3333333333333333</v>
       </c>
     </row>
     <row r="77">
@@ -6684,22 +6706,22 @@
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>Parral</t>
+          <t>Linares</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>Hospital San José (Parral)</t>
+          <t>Hospital Presidente Carlos Ibáñez del Campo (Linares)</t>
         </is>
       </c>
       <c r="E77" s="3" t="n">
-        <v>71</v>
+        <v>1194</v>
       </c>
       <c r="F77" s="3" t="n">
-        <v>108</v>
+        <v>1437</v>
       </c>
       <c r="G77" s="4" t="n">
-        <v>0.6574074074074074</v>
+        <v>0.8308977035490606</v>
       </c>
     </row>
     <row r="78">
@@ -6715,22 +6737,22 @@
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>San Javier</t>
+          <t>Parral</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>Hospital Dr. Abel Fuentealba Lagos de San Javier</t>
+          <t>Hospital San José (Parral)</t>
         </is>
       </c>
       <c r="E78" s="3" t="n">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="F78" s="3" t="n">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="G78" s="4" t="n">
-        <v>0.78</v>
+        <v>0.7592592592592593</v>
       </c>
     </row>
     <row r="79">
@@ -6746,53 +6768,53 @@
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>Talca</t>
+          <t>San Javier</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>Hospital Dr. César Garavagno Burotto (Talca)</t>
+          <t>Hospital Dr. Abel Fuentealba Lagos de San Javier</t>
         </is>
       </c>
       <c r="E79" s="3" t="n">
-        <v>3307</v>
+        <v>87</v>
       </c>
       <c r="F79" s="3" t="n">
-        <v>3615</v>
+        <v>100</v>
       </c>
       <c r="G79" s="4" t="n">
-        <v>0.9147994467496542</v>
+        <v>0.87</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>Metropolitana de Santiago</t>
+          <t>Maule</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>Servicio de Salud Metropolitano Central</t>
+          <t>Servicio de Salud Del Maule</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>Maipú</t>
+          <t>Talca</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>Hospital Clínico Metropolitano El Carmen Doctor Luis Valentín Ferrada</t>
+          <t>Hospital Dr. César Garavagno Burotto (Talca)</t>
         </is>
       </c>
       <c r="E80" s="3" t="n">
-        <v>2197</v>
+        <v>3347</v>
       </c>
       <c r="F80" s="3" t="n">
-        <v>2305</v>
+        <v>3615</v>
       </c>
       <c r="G80" s="4" t="n">
-        <v>0.9531453362255965</v>
+        <v>0.9258644536652836</v>
       </c>
     </row>
     <row r="81">
@@ -6808,22 +6830,22 @@
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>Santiago</t>
+          <t>Maipú</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>Hospital Clínico San Borja Arriarán</t>
+          <t>Hospital Clínico Metropolitano El Carmen Doctor Luis Valentín Ferrada</t>
         </is>
       </c>
       <c r="E81" s="3" t="n">
-        <v>2764</v>
+        <v>2197</v>
       </c>
       <c r="F81" s="3" t="n">
-        <v>3028</v>
+        <v>2305</v>
       </c>
       <c r="G81" s="4" t="n">
-        <v>0.9128137384412153</v>
+        <v>0.9531453362255965</v>
       </c>
     </row>
     <row r="82">
@@ -6834,27 +6856,27 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>Servicio de Salud Metropolitano Norte</t>
+          <t>Servicio de Salud Metropolitano Central</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>Colina</t>
+          <t>Santiago</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>SAPU Esmeralda</t>
+          <t>Hospital Clínico San Borja Arriarán</t>
         </is>
       </c>
       <c r="E82" s="3" t="n">
-        <v>1</v>
+        <v>2764</v>
       </c>
       <c r="F82" s="3" t="n">
-        <v>1</v>
+        <v>3028</v>
       </c>
       <c r="G82" s="4" t="n">
-        <v>1</v>
+        <v>0.9128137384412153</v>
       </c>
     </row>
     <row r="83">
@@ -6875,17 +6897,17 @@
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>SAR Colina</t>
+          <t>SAPU Esmeralda</t>
         </is>
       </c>
       <c r="E83" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F83" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G83" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="84">
@@ -6901,22 +6923,22 @@
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>Independencia</t>
+          <t>Colina</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>Complejo Hospitalario San José (Santiago, Independencia)</t>
+          <t>SAR Colina</t>
         </is>
       </c>
       <c r="E84" s="3" t="n">
-        <v>3774</v>
+        <v>2</v>
       </c>
       <c r="F84" s="3" t="n">
-        <v>4480</v>
+        <v>1</v>
       </c>
       <c r="G84" s="4" t="n">
-        <v>0.8424107142857142</v>
+        <v>2</v>
       </c>
     </row>
     <row r="85">
@@ -6927,27 +6949,27 @@
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>Servicio de Salud Metropolitano Occidente</t>
+          <t>Servicio de Salud Metropolitano Norte</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>Cerro Navia</t>
+          <t>Independencia</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>Hospital  Félix Bulnes Cerda</t>
+          <t>Complejo Hospitalario San José (Santiago, Independencia)</t>
         </is>
       </c>
       <c r="E85" s="3" t="n">
-        <v>2296</v>
+        <v>4148</v>
       </c>
       <c r="F85" s="3" t="n">
-        <v>2621</v>
+        <v>4480</v>
       </c>
       <c r="G85" s="4" t="n">
-        <v>0.876001526135063</v>
+        <v>0.9258928571428572</v>
       </c>
     </row>
     <row r="86">
@@ -6963,22 +6985,22 @@
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>Curacaví</t>
+          <t>Cerro Navia</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>Hospital de Curacaví</t>
+          <t>Hospital  Félix Bulnes Cerda</t>
         </is>
       </c>
       <c r="E86" s="3" t="n">
-        <v>0</v>
+        <v>2418</v>
       </c>
       <c r="F86" s="3" t="n">
-        <v>1</v>
+        <v>2621</v>
       </c>
       <c r="G86" s="4" t="n">
-        <v>0</v>
+        <v>0.9225486455551316</v>
       </c>
     </row>
     <row r="87">
@@ -6994,22 +7016,22 @@
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>Melipilla</t>
+          <t>Curacaví</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>Hospital San José (Melipilla)</t>
+          <t>Hospital de Curacaví</t>
         </is>
       </c>
       <c r="E87" s="3" t="n">
-        <v>1281</v>
+        <v>0</v>
       </c>
       <c r="F87" s="3" t="n">
-        <v>1484</v>
+        <v>1</v>
       </c>
       <c r="G87" s="4" t="n">
-        <v>0.8632075471698113</v>
+        <v>0</v>
       </c>
     </row>
     <row r="88">
@@ -7025,22 +7047,22 @@
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>Peñaflor</t>
+          <t>Melipilla</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>Hospital de Peñaflor</t>
+          <t>Hospital San José (Melipilla)</t>
         </is>
       </c>
       <c r="E88" s="3" t="n">
-        <v>52</v>
+        <v>1281</v>
       </c>
       <c r="F88" s="3" t="n">
-        <v>62</v>
+        <v>1484</v>
       </c>
       <c r="G88" s="4" t="n">
-        <v>0.8387096774193549</v>
+        <v>0.8632075471698113</v>
       </c>
     </row>
     <row r="89">
@@ -7056,22 +7078,22 @@
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>Santiago</t>
+          <t>Peñaflor</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>Hospital San Juan de Dios (Santiago, Santiago)</t>
+          <t>Hospital de Peñaflor</t>
         </is>
       </c>
       <c r="E89" s="3" t="n">
-        <v>1983</v>
+        <v>52</v>
       </c>
       <c r="F89" s="3" t="n">
-        <v>2072</v>
+        <v>62</v>
       </c>
       <c r="G89" s="4" t="n">
-        <v>0.957046332046332</v>
+        <v>0.8387096774193549</v>
       </c>
     </row>
     <row r="90">
@@ -7087,22 +7109,22 @@
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>Talagante</t>
+          <t>Santiago</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>Hospital Adalberto Steeger (Talagante)</t>
+          <t>Hospital San Juan de Dios (Santiago, Santiago)</t>
         </is>
       </c>
       <c r="E90" s="3" t="n">
-        <v>547</v>
+        <v>2077</v>
       </c>
       <c r="F90" s="3" t="n">
-        <v>825</v>
+        <v>2072</v>
       </c>
       <c r="G90" s="4" t="n">
-        <v>0.6630303030303031</v>
+        <v>1.002413127413127</v>
       </c>
     </row>
     <row r="91">
@@ -7113,27 +7135,27 @@
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>Servicio de Salud Metropolitano Oriente</t>
+          <t>Servicio de Salud Metropolitano Occidente</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>Peñalolén</t>
+          <t>Talagante</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>Hospital Dr. Luis Tisné B. (Santiago, Peñalolén)</t>
+          <t>Hospital Adalberto Steeger (Talagante)</t>
         </is>
       </c>
       <c r="E91" s="3" t="n">
-        <v>2559</v>
+        <v>809</v>
       </c>
       <c r="F91" s="3" t="n">
-        <v>2814</v>
+        <v>825</v>
       </c>
       <c r="G91" s="4" t="n">
-        <v>0.9093816631130064</v>
+        <v>0.9806060606060606</v>
       </c>
     </row>
     <row r="92">
@@ -7144,27 +7166,27 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>Servicio de Salud Metropolitano Sur</t>
+          <t>Servicio de Salud Metropolitano Oriente</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>San Bernardo</t>
+          <t>Peñalolén</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>Hospital El Pino (Santiago, San Bernardo)</t>
+          <t>Hospital Dr. Luis Tisné B. (Santiago, Peñalolén)</t>
         </is>
       </c>
       <c r="E92" s="3" t="n">
-        <v>1544</v>
+        <v>2613</v>
       </c>
       <c r="F92" s="3" t="n">
-        <v>1629</v>
+        <v>2814</v>
       </c>
       <c r="G92" s="4" t="n">
-        <v>0.9478207489257213</v>
+        <v>0.9285714285714286</v>
       </c>
     </row>
     <row r="93">
@@ -7185,17 +7207,17 @@
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>Hospital Parroquial de San Bernardo (D)</t>
+          <t>Hospital El Pino (Santiago, San Bernardo)</t>
         </is>
       </c>
       <c r="E93" s="3" t="n">
-        <v>1269</v>
+        <v>1571</v>
       </c>
       <c r="F93" s="3" t="n">
-        <v>1309</v>
+        <v>1629</v>
       </c>
       <c r="G93" s="4" t="n">
-        <v>0.9694423223834988</v>
+        <v>0.9643953345610804</v>
       </c>
     </row>
     <row r="94">
@@ -7206,27 +7228,27 @@
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>Servicio de Salud Metropolitano Sur Oriente</t>
+          <t>Servicio de Salud Metropolitano Sur</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>La Florida</t>
+          <t>San Bernardo</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>Hospital Clínico Metropolitano La Florida Dra. Eloísa Díaz Insunza</t>
+          <t>Hospital Parroquial de San Bernardo (D)</t>
         </is>
       </c>
       <c r="E94" s="3" t="n">
-        <v>1899</v>
+        <v>1280</v>
       </c>
       <c r="F94" s="3" t="n">
-        <v>2045</v>
+        <v>1309</v>
       </c>
       <c r="G94" s="4" t="n">
-        <v>0.9286063569682151</v>
+        <v>0.9778456837280367</v>
       </c>
     </row>
     <row r="95">
@@ -7242,22 +7264,22 @@
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>Puente Alto</t>
+          <t>La Florida</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>Complejo Hospitalario Dr. Sótero del Río (Santiago, Puente Alto)</t>
+          <t>Hospital Clínico Metropolitano La Florida Dra. Eloísa Díaz Insunza</t>
         </is>
       </c>
       <c r="E95" s="3" t="n">
-        <v>2261</v>
+        <v>1908</v>
       </c>
       <c r="F95" s="3" t="n">
-        <v>2941</v>
+        <v>2045</v>
       </c>
       <c r="G95" s="4" t="n">
-        <v>0.7687861271676301</v>
+        <v>0.9330073349633252</v>
       </c>
     </row>
     <row r="96">
@@ -7273,52 +7295,54 @@
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>San Ramón</t>
+          <t>Puente Alto</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>Hospital Padre Alberto Hurtado (San Ramón)</t>
+          <t>Complejo Hospitalario Dr. Sótero del Río (Santiago, Puente Alto)</t>
         </is>
       </c>
       <c r="E96" s="3" t="n">
-        <v>1635</v>
+        <v>2297</v>
       </c>
       <c r="F96" s="3" t="n">
-        <v>1854</v>
+        <v>2941</v>
       </c>
       <c r="G96" s="4" t="n">
-        <v>0.8818770226537217</v>
+        <v>0.7810268616116967</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>Tarapacá</t>
+          <t>Metropolitana de Santiago</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>Servicio de Salud Tarapacá</t>
+          <t>Servicio de Salud Metropolitano Sur Oriente</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>Alto Hospicio</t>
+          <t>San Ramón</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>Centro de Salud Familiar Pedro Pulgar Melgarejo</t>
+          <t>Hospital Padre Alberto Hurtado (San Ramón)</t>
         </is>
       </c>
       <c r="E97" s="3" t="n">
-        <v>7</v>
+        <v>1671</v>
       </c>
       <c r="F97" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G97" s="4" t="n"/>
+        <v>1854</v>
+      </c>
+      <c r="G97" s="4" t="n">
+        <v>0.901294498381877</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -7338,18 +7362,16 @@
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>Hospital de Alto Hospicio</t>
+          <t>Centro de Salud Familiar Pedro Pulgar Melgarejo</t>
         </is>
       </c>
       <c r="E98" s="3" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="F98" s="3" t="n">
-        <v>21</v>
-      </c>
-      <c r="G98" s="4" t="n">
-        <v>0.5714285714285714</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G98" s="4" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -7364,53 +7386,53 @@
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>Iquique</t>
+          <t>Alto Hospicio</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>Hospital Dr. Ernesto Torres Galdames (Iquique)</t>
+          <t>Hospital de Alto Hospicio</t>
         </is>
       </c>
       <c r="E99" s="3" t="n">
-        <v>2036</v>
+        <v>16</v>
       </c>
       <c r="F99" s="3" t="n">
-        <v>3192</v>
+        <v>21</v>
       </c>
       <c r="G99" s="4" t="n">
-        <v>0.6378446115288221</v>
+        <v>0.7619047619047619</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>Valparaíso</t>
+          <t>Tarapacá</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>Servicio de Salud Aconcagua</t>
+          <t>Servicio de Salud Tarapacá</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>Llaillay</t>
+          <t>Iquique</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>Hospital San Francisco (Llaillay)</t>
+          <t>Hospital Dr. Ernesto Torres Galdames (Iquique)</t>
         </is>
       </c>
       <c r="E100" s="3" t="n">
-        <v>0</v>
+        <v>2175</v>
       </c>
       <c r="F100" s="3" t="n">
-        <v>1</v>
+        <v>3192</v>
       </c>
       <c r="G100" s="4" t="n">
-        <v>0</v>
+        <v>0.681390977443609</v>
       </c>
     </row>
     <row r="101">
@@ -7426,22 +7448,22 @@
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>Los Andes</t>
+          <t>Llaillay</t>
         </is>
       </c>
       <c r="D101" s="2" t="inlineStr">
         <is>
-          <t>Hospital San Juan de Dios (Los Andes)</t>
+          <t>Hospital San Francisco (Llaillay)</t>
         </is>
       </c>
       <c r="E101" s="3" t="n">
-        <v>627</v>
+        <v>1</v>
       </c>
       <c r="F101" s="3" t="n">
-        <v>637</v>
+        <v>1</v>
       </c>
       <c r="G101" s="4" t="n">
-        <v>0.9843014128728415</v>
+        <v>1</v>
       </c>
     </row>
     <row r="102">
@@ -7457,22 +7479,22 @@
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>San Felipe</t>
+          <t>Los Andes</t>
         </is>
       </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t>Hospital San Camilo de San Felipe</t>
+          <t>Hospital San Juan de Dios (Los Andes)</t>
         </is>
       </c>
       <c r="E102" s="3" t="n">
-        <v>1049</v>
+        <v>630</v>
       </c>
       <c r="F102" s="3" t="n">
-        <v>1262</v>
+        <v>637</v>
       </c>
       <c r="G102" s="4" t="n">
-        <v>0.8312202852614897</v>
+        <v>0.9890109890109891</v>
       </c>
     </row>
     <row r="103">
@@ -7483,27 +7505,27 @@
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>Servicio de Salud Metropolitano Oriente</t>
+          <t>Servicio de Salud Aconcagua</t>
         </is>
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>Isla de Pascua</t>
+          <t>San Felipe</t>
         </is>
       </c>
       <c r="D103" s="2" t="inlineStr">
         <is>
-          <t>Hospital Hanga Roa (Isla De Pascua)</t>
+          <t>Hospital San Camilo de San Felipe</t>
         </is>
       </c>
       <c r="E103" s="3" t="n">
-        <v>76</v>
+        <v>1116</v>
       </c>
       <c r="F103" s="3" t="n">
-        <v>86</v>
+        <v>1262</v>
       </c>
       <c r="G103" s="4" t="n">
-        <v>0.8837209302325582</v>
+        <v>0.884310618066561</v>
       </c>
     </row>
     <row r="104">
@@ -7514,27 +7536,27 @@
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>Servicio de Salud Valparaíso San Antonio</t>
+          <t>Servicio de Salud Metropolitano Oriente</t>
         </is>
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>San Antonio</t>
+          <t>Isla de Pascua</t>
         </is>
       </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t>Hospital Claudio Vicuña (San Antonio)</t>
+          <t>Hospital Hanga Roa (Isla De Pascua)</t>
         </is>
       </c>
       <c r="E104" s="3" t="n">
-        <v>538</v>
+        <v>81</v>
       </c>
       <c r="F104" s="3" t="n">
-        <v>1038</v>
+        <v>86</v>
       </c>
       <c r="G104" s="4" t="n">
-        <v>0.5183044315992292</v>
+        <v>0.9418604651162791</v>
       </c>
     </row>
     <row r="105">
@@ -7550,22 +7572,22 @@
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>Valparaíso</t>
+          <t>San Antonio</t>
         </is>
       </c>
       <c r="D105" s="2" t="inlineStr">
         <is>
-          <t>Hospital Carlos Van Buren (Valparaíso)</t>
+          <t>Hospital Claudio Vicuña (San Antonio)</t>
         </is>
       </c>
       <c r="E105" s="3" t="n">
-        <v>1246</v>
+        <v>548</v>
       </c>
       <c r="F105" s="3" t="n">
-        <v>1377</v>
+        <v>1038</v>
       </c>
       <c r="G105" s="4" t="n">
-        <v>0.9048656499636892</v>
+        <v>0.5279383429672447</v>
       </c>
     </row>
     <row r="106">
@@ -7576,58 +7598,58 @@
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>Servicio de Salud Viña del Mar Quillota</t>
+          <t>Servicio de Salud Valparaíso San Antonio</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>Quintero</t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
-          <t>Hospital Adriana Cousiño (Quintero)</t>
+          <t>Hospital Carlos Van Buren (Valparaíso)</t>
         </is>
       </c>
       <c r="E106" s="3" t="n">
-        <v>1</v>
+        <v>1258</v>
       </c>
       <c r="F106" s="3" t="n">
-        <v>1</v>
+        <v>1377</v>
       </c>
       <c r="G106" s="4" t="n">
-        <v>1</v>
+        <v>0.9135802469135802</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>Ñuble</t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>Servicio de Salud Ñuble</t>
+          <t>Servicio de Salud Viña del Mar Quillota</t>
         </is>
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>Bulnes</t>
+          <t>Quintero</t>
         </is>
       </c>
       <c r="D107" s="2" t="inlineStr">
         <is>
-          <t>Hospital Comunitario de Salud Familiar de Bulnes</t>
+          <t>Hospital Adriana Cousiño (Quintero)</t>
         </is>
       </c>
       <c r="E107" s="3" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F107" s="3" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G107" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="108">
@@ -7643,22 +7665,22 @@
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>Chillán</t>
+          <t>Bulnes</t>
         </is>
       </c>
       <c r="D108" s="2" t="inlineStr">
         <is>
-          <t>Hospital Clínico Herminda Martín (Chillán)</t>
+          <t>Hospital Comunitario de Salud Familiar de Bulnes</t>
         </is>
       </c>
       <c r="E108" s="3" t="n">
-        <v>1544</v>
+        <v>5</v>
       </c>
       <c r="F108" s="3" t="n">
-        <v>1934</v>
+        <v>5</v>
       </c>
       <c r="G108" s="4" t="n">
-        <v>0.7983453981385729</v>
+        <v>1</v>
       </c>
     </row>
     <row r="109">
@@ -7674,22 +7696,22 @@
       </c>
       <c r="C109" s="2" t="inlineStr">
         <is>
-          <t>Coelemu</t>
+          <t>Chillán</t>
         </is>
       </c>
       <c r="D109" s="2" t="inlineStr">
         <is>
-          <t>Hospital Comunitario de Salud Familiar Dr. Eduardo Contreras Trabucco de Coelemu</t>
+          <t>Hospital Clínico Herminda Martín (Chillán)</t>
         </is>
       </c>
       <c r="E109" s="3" t="n">
-        <v>1</v>
+        <v>1748</v>
       </c>
       <c r="F109" s="3" t="n">
-        <v>2</v>
+        <v>1934</v>
       </c>
       <c r="G109" s="4" t="n">
-        <v>0.5</v>
+        <v>0.9038262668045501</v>
       </c>
     </row>
     <row r="110">
@@ -7705,22 +7727,22 @@
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>El Carmen</t>
+          <t>Coelemu</t>
         </is>
       </c>
       <c r="D110" s="2" t="inlineStr">
         <is>
-          <t>Hospital Comunitario de Salud Familiar de El Carmen</t>
+          <t>Hospital Comunitario de Salud Familiar Dr. Eduardo Contreras Trabucco de Coelemu</t>
         </is>
       </c>
       <c r="E110" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F110" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G110" s="4" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="111">
@@ -7736,22 +7758,22 @@
       </c>
       <c r="C111" s="2" t="inlineStr">
         <is>
-          <t>Quirihue</t>
+          <t>El Carmen</t>
         </is>
       </c>
       <c r="D111" s="2" t="inlineStr">
         <is>
-          <t>Hospital Comunitario de Salud Familiar de Quirihue</t>
+          <t>Hospital Comunitario de Salud Familiar de El Carmen</t>
         </is>
       </c>
       <c r="E111" s="3" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F111" s="3" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="G111" s="4" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="112">
@@ -7767,22 +7789,22 @@
       </c>
       <c r="C112" s="2" t="inlineStr">
         <is>
-          <t>San Carlos</t>
+          <t>Quirihue</t>
         </is>
       </c>
       <c r="D112" s="2" t="inlineStr">
         <is>
-          <t>Hospital de San Carlos</t>
+          <t>Hospital Comunitario de Salud Familiar de Quirihue</t>
         </is>
       </c>
       <c r="E112" s="3" t="n">
-        <v>526</v>
+        <v>3</v>
       </c>
       <c r="F112" s="3" t="n">
-        <v>538</v>
+        <v>6</v>
       </c>
       <c r="G112" s="4" t="n">
-        <v>0.9776951672862454</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="113">
@@ -7798,26 +7820,57 @@
       </c>
       <c r="C113" s="2" t="inlineStr">
         <is>
+          <t>San Carlos</t>
+        </is>
+      </c>
+      <c r="D113" s="2" t="inlineStr">
+        <is>
+          <t>Hospital de San Carlos</t>
+        </is>
+      </c>
+      <c r="E113" s="3" t="n">
+        <v>742</v>
+      </c>
+      <c r="F113" s="3" t="n">
+        <v>538</v>
+      </c>
+      <c r="G113" s="4" t="n">
+        <v>1.379182156133829</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="inlineStr">
+        <is>
+          <t>Ñuble</t>
+        </is>
+      </c>
+      <c r="B114" s="2" t="inlineStr">
+        <is>
+          <t>Servicio de Salud Ñuble</t>
+        </is>
+      </c>
+      <c r="C114" s="2" t="inlineStr">
+        <is>
           <t>Yungay</t>
         </is>
       </c>
-      <c r="D113" s="2" t="inlineStr">
+      <c r="D114" s="2" t="inlineStr">
         <is>
           <t>Hospital Comunitario de Salud Familiar Pedro Morales Campos (Yungay)</t>
         </is>
       </c>
-      <c r="E113" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F113" s="3" t="n">
+      <c r="E114" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="G113" s="4" t="n">
-        <v>0</v>
+      <c r="F114" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G114" s="4" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G113"/>
+  <autoFilter ref="A1:G114"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>